<commit_message>
tanda tangan footer OSH, Manager, HRD
</commit_message>
<xml_diff>
--- a/src/templates/Footer_Form_Absen.xlsx
+++ b/src/templates/Footer_Form_Absen.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tomat/Documents/Projek Mobile App/apiAbsen/src/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF3001A5-D510-8449-933F-5ACC7A5D2688}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B25025C4-27F5-AF46-AA62-5C7B537D28BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="19960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="TTD_TEMPLATE" sheetId="6" state="hidden" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'TEMPLATE 1'!$A$1:$J$13</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'TEMPLATE 1'!$A$1:$J$12</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -112,12 +112,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2191,14 +2194,14 @@
       <c r="Y6" s="2"/>
       <c r="Z6" s="2"/>
     </row>
-    <row r="7" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
+    <row r="7" spans="1:26" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="5"/>
+      <c r="B7" s="5"/>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
+      <c r="F7" s="5"/>
+      <c r="G7" s="5"/>
       <c r="H7" s="3"/>
       <c r="I7" s="1"/>
       <c r="J7" s="1"/>
@@ -2219,13 +2222,13 @@
       <c r="Z7" s="2"/>
     </row>
     <row r="8" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
+      <c r="A8" s="5"/>
+      <c r="B8" s="5"/>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
+      <c r="F8" s="5"/>
+      <c r="G8" s="5"/>
       <c r="H8" s="3"/>
       <c r="I8" s="1"/>
       <c r="J8" s="1"/>
@@ -2251,7 +2254,9 @@
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
+      <c r="F9" s="4" t="s">
+        <v>5</v>
+      </c>
       <c r="G9" s="2"/>
       <c r="H9" s="3"/>
       <c r="I9" s="1"/>
@@ -2278,7 +2283,9 @@
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
+      <c r="F10" s="2" t="s">
+        <v>6</v>
+      </c>
       <c r="G10" s="2"/>
       <c r="H10" s="3"/>
       <c r="I10" s="1"/>
@@ -2299,7 +2306,7 @@
       <c r="Y10" s="2"/>
       <c r="Z10" s="2"/>
     </row>
-    <row r="11" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:26" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -2315,9 +2322,6 @@
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
-      <c r="F12" s="4" t="s">
-        <v>5</v>
-      </c>
       <c r="G12" s="2"/>
       <c r="H12" s="3"/>
     </row>
@@ -2327,13 +2331,16 @@
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
-      <c r="F13" s="2" t="s">
-        <v>6</v>
-      </c>
       <c r="G13" s="2"/>
       <c r="H13" s="3"/>
     </row>
   </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="F7:G7"/>
+  </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0.3" footer="0.3"/>
   <pageSetup paperSize="14" scale="86" fitToHeight="0" orientation="portrait"/>

</xml_diff>

<commit_message>
update footer & list_users
</commit_message>
<xml_diff>
--- a/src/templates/Footer_Form_Absen.xlsx
+++ b/src/templates/Footer_Form_Absen.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tomat/Documents/Projek Mobile App/apiAbsen/src/templates/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tomat/Developer/apiAbsen/src/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B25025C4-27F5-AF46-AA62-5C7B537D28BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2461BE8A-2E9D-CE46-BC91-223CA2B9DEC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="19960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="8">
   <si>
     <t>Note :</t>
   </si>
@@ -58,6 +58,9 @@
   </si>
   <si>
     <t>PIC Approval 1</t>
+  </si>
+  <si>
+    <t>Dicek Oleh,</t>
   </si>
 </sst>
 </file>
@@ -2280,7 +2283,9 @@
     <row r="10" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
+      <c r="C10" s="2" t="s">
+        <v>7</v>
+      </c>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
       <c r="F10" s="2" t="s">

</xml_diff>

<commit_message>
Tambahan Jabatan Pada HRD
</commit_message>
<xml_diff>
--- a/src/templates/Footer_Form_Absen.xlsx
+++ b/src/templates/Footer_Form_Absen.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tomat/Developer/apiAbsen/src/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2461BE8A-2E9D-CE46-BC91-223CA2B9DEC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72E59E26-6560-E44E-AEA4-901020893E8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="19960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="TTD_TEMPLATE" sheetId="6" state="hidden" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'TEMPLATE 1'!$A$1:$J$12</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'TEMPLATE 1'!$A$1:$J$13</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>

</xml_diff>